<commit_message>
Fix damaged file: replace treemap XML injection with native openpyxl BarCharts
</commit_message>
<xml_diff>
--- a/SX_Steady_State_Model_26elem.xlsx
+++ b/SX_Steady_State_Model_26elem.xlsx
@@ -552,6 +552,244 @@
                 </a:pPr>
                 <a:r>
                   <a:t>LN(D)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Raffinate Concentration — 26 Elements (g/L)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'SX Model'!C289</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="B71C1C"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="B71C1C"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'SX Model'!$A$290:$A$315</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'SX Model'!$C$290:$C$315</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Element</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Concentration (g/L)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Pregnant Solution — 26 Elements (g/L)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'SX Model'!D289</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="1B5E20"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="1B5E20"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'SX Model'!$A$290:$A$315</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'SX Model'!$D$290:$D$315</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Element</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Concentration (g/L)</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -1515,154 +1753,123 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
-<cx:chartSpace xmlns:cx="http://schemas.microsoft.com/office/drawing/2016/5/9/chartex" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <cx:chartData>
-    <cx:externalData r:id="rId1"/>
-    <cx:data id="0">
-      <cx:strDim type="cat">
-        <cx:f>'SX Model'!$E$290:$E$315</cx:f>
-      </cx:strDim>
-      <cx:strDim type="cat">
-        <cx:f>'SX Model'!$A$290:$A$315</cx:f>
-      </cx:strDim>
-      <cx:numDim type="val">
-        <cx:f>'SX Model'!$B$290:$B$315</cx:f>
-      </cx:numDim>
-    </cx:data>
-  </cx:chartData>
-  <cx:chart>
-    <cx:title overlay="0">
-      <cx:tx>
-        <cx:rich>
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
           <a:bodyPr/>
-          <a:lstStyle/>
           <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
             <a:r>
-              <a:t>Feed Concentration (g/L) — 26 Elements</a:t>
+              <a:t>Feed Concentration — 26 Elements (g/L)</a:t>
             </a:r>
           </a:p>
-        </cx:rich>
-      </cx:tx>
-    </cx:title>
-    <cx:plotArea>
-      <cx:plotAreaRegion>
-        <cx:series layoutId="treemap" ownsLabel="1" formatIdx="0" uniqueId="{00000000-0000-0000-0000-000000000002}">
-          <cx:dataId val="0"/>
-          <cx:layoutPr>
-            <cx:visibility headerSelect="1" outlineSelect="1"/>
-          </cx:layoutPr>
-        </cx:series>
-      </cx:plotAreaRegion>
-    </cx:plotArea>
-    <cx:legend>
-      <cx:visibility val="0"/>
-    </cx:legend>
-  </cx:chart>
-  <cx:clrMapOvr>
-    <a:overrideClrMapping/>
-  </cx:clrMapOvr>
-</cx:chartSpace>
-</file>
-
-<file path=xl/charts/chartEx2.xml><?xml version="1.0" encoding="utf-8"?>
-<cx:chartSpace xmlns:cx="http://schemas.microsoft.com/office/drawing/2016/5/9/chartex" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <cx:chartData>
-    <cx:externalData r:id="rId1"/>
-    <cx:data id="0">
-      <cx:strDim type="cat">
-        <cx:f>'SX Model'!$E$290:$E$315</cx:f>
-      </cx:strDim>
-      <cx:strDim type="cat">
-        <cx:f>'SX Model'!$A$290:$A$315</cx:f>
-      </cx:strDim>
-      <cx:numDim type="val">
-        <cx:f>'SX Model'!$C$290:$C$315</cx:f>
-      </cx:numDim>
-    </cx:data>
-  </cx:chartData>
-  <cx:chart>
-    <cx:title overlay="0">
-      <cx:tx>
-        <cx:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:r>
-              <a:t>Raffinate Concentration (g/L) — 26 Elements</a:t>
-            </a:r>
-          </a:p>
-        </cx:rich>
-      </cx:tx>
-    </cx:title>
-    <cx:plotArea>
-      <cx:plotAreaRegion>
-        <cx:series layoutId="treemap" ownsLabel="1" formatIdx="0" uniqueId="{00000000-0000-0000-0000-000000000003}">
-          <cx:dataId val="0"/>
-          <cx:layoutPr>
-            <cx:visibility headerSelect="1" outlineSelect="1"/>
-          </cx:layoutPr>
-        </cx:series>
-      </cx:plotAreaRegion>
-    </cx:plotArea>
-    <cx:legend>
-      <cx:visibility val="0"/>
-    </cx:legend>
-  </cx:chart>
-  <cx:clrMapOvr>
-    <a:overrideClrMapping/>
-  </cx:clrMapOvr>
-</cx:chartSpace>
-</file>
-
-<file path=xl/charts/chartEx3.xml><?xml version="1.0" encoding="utf-8"?>
-<cx:chartSpace xmlns:cx="http://schemas.microsoft.com/office/drawing/2016/5/9/chartex" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <cx:chartData>
-    <cx:externalData r:id="rId1"/>
-    <cx:data id="0">
-      <cx:strDim type="cat">
-        <cx:f>'SX Model'!$E$290:$E$315</cx:f>
-      </cx:strDim>
-      <cx:strDim type="cat">
-        <cx:f>'SX Model'!$A$290:$A$315</cx:f>
-      </cx:strDim>
-      <cx:numDim type="val">
-        <cx:f>'SX Model'!$D$290:$D$315</cx:f>
-      </cx:numDim>
-    </cx:data>
-  </cx:chartData>
-  <cx:chart>
-    <cx:title overlay="0">
-      <cx:tx>
-        <cx:rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:r>
-              <a:t>Pregnant Solution (g/L) — 26 Elements</a:t>
-            </a:r>
-          </a:p>
-        </cx:rich>
-      </cx:tx>
-    </cx:title>
-    <cx:plotArea>
-      <cx:plotAreaRegion>
-        <cx:series layoutId="treemap" ownsLabel="1" formatIdx="0" uniqueId="{00000000-0000-0000-0000-000000000004}">
-          <cx:dataId val="0"/>
-          <cx:layoutPr>
-            <cx:visibility headerSelect="1" outlineSelect="1"/>
-          </cx:layoutPr>
-        </cx:series>
-      </cx:plotAreaRegion>
-    </cx:plotArea>
-    <cx:legend>
-      <cx:visibility val="0"/>
-    </cx:legend>
-  </cx:chart>
-  <cx:clrMapOvr>
-    <a:overrideClrMapping/>
-  </cx:clrMapOvr>
-</cx:chartSpace>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'SX Model'!B289</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="1B3A6B"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="1B3A6B"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'SX Model'!$A$290:$A$315</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'SX Model'!$B$290:$B$315</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Element</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Concentration (g/L)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1848,102 +2055,73 @@
     </graphicFrame>
     <clientData/>
   </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor moveWithCells="1">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>318</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>348</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart"/>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>318</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10080000" cy="5040000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="5" name="Chart 5"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="rId1"/>
+          <c:chart r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor moveWithCells="1">
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>318</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>348</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart"/>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>350</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10080000" cy="5040000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="6" name="Chart 6"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="rId2"/>
+          <c:chart r:id="rId6"/>
         </a:graphicData>
       </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor moveWithCells="1">
-    <xdr:from>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>318</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>348</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart"/>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>382</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10080000" cy="5040000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="7" name="Chart 7"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="rId3"/>
+          <c:chart r:id="rId7"/>
         </a:graphicData>
       </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2230,7 +2408,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002E7D32"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7449,7 +7627,6 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -38580,7 +38757,7 @@
     <row r="288" ht="18" customHeight="1">
       <c r="A288" s="13" t="inlineStr">
         <is>
-          <t>TREEMAP DATA — Feed / Raffinate / Pregnant  (g/L)  → rendered as Treemap charts in Excel 2016+</t>
+          <t>ELEMENT CONCENTRATION DATA — Feed / Raffinate / Pregnant  (g/L)</t>
         </is>
       </c>
     </row>
@@ -39263,6 +39440,7 @@
     <mergeCell ref="A1:BZ1"/>
     <mergeCell ref="EH89:EO89"/>
     <mergeCell ref="GL89:GS89"/>
+    <mergeCell ref="A288:AB288"/>
     <mergeCell ref="HO89:HO90"/>
     <mergeCell ref="A89:A90"/>
     <mergeCell ref="HL89:HL90"/>
@@ -39285,7 +39463,6 @@
     <mergeCell ref="HV89:HV90"/>
     <mergeCell ref="IA89:IA90"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A288:AA288"/>
     <mergeCell ref="AP89:AW89"/>
     <mergeCell ref="HG89:HG90"/>
     <mergeCell ref="HB89:HB90"/>

</xml_diff>